<commit_message>
criação grafico e ajustes pontuais
</commit_message>
<xml_diff>
--- a/src/testeHttp/FALTAS.xlsx
+++ b/src/testeHttp/FALTAS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/62180101100c7fdd/Desktop/backend-gestao-faltas/src/testeHttp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="38" documentId="13_ncr:1_{22835482-9EB8-410C-9085-30BFCD91445F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A80844C3-F852-4703-A562-3F6B05B58127}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="13_ncr:1_{22835482-9EB8-410C-9085-30BFCD91445F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5B0CDEF-D5E7-4071-93ED-8256691EC610}"/>
   <bookViews>
     <workbookView xWindow="4428" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{50DC5498-AC41-49C0-9C02-4449CC76D463}"/>
   </bookViews>
@@ -608,7 +608,7 @@
         <v>0</v>
       </c>
       <c r="E11">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
@@ -642,7 +642,7 @@
         <v>0</v>
       </c>
       <c r="E13">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
@@ -676,7 +676,7 @@
         <v>0</v>
       </c>
       <c r="E15">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>